<commit_message>
Made some new changes to the TestLab IP Config...
 Changes to be committed:
	modified:   TestLab IP Configuration.xlsx

	Noteworthy changes to TestLab IP Configuration.xlsx
	1. Made slight changes to some of the IP Address Ranges.
	2. Added a column which tracks the # of potential hosts
	   in a particular DHCP IP Range.
	3. Addded a sum function for the column in item #2 to show
	   the total number of IP addresses in all of the different
	    IP range sections listed on the IP Address Range chart
	   for the Homeone Test Lab Subnet.
	4. Made some minor color improvements to the Excel charts.
</commit_message>
<xml_diff>
--- a/TestLab IP Configuration.xlsx
+++ b/TestLab IP Configuration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{956B7102-1419-4FAB-B15E-9F59E6367E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A5BDCE-BC53-4FFE-981D-6A319B84E0E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
   <si>
     <t>Testlab Network:</t>
   </si>
@@ -93,9 +92,6 @@
     <t>IP Range By Color</t>
   </si>
   <si>
-    <t>10.0.2.21 - 10.0.2.91</t>
-  </si>
-  <si>
     <t>10.0.2.91 - 10.0.2.99</t>
   </si>
   <si>
@@ -141,18 +137,9 @@
     <t>10.0.2.252</t>
   </si>
   <si>
-    <t>Hole-RPSV PiHole/DNS Srv</t>
-  </si>
-  <si>
     <t>10.0.2.254</t>
   </si>
   <si>
-    <t>10.0.2.200 - 10.0.2.254</t>
-  </si>
-  <si>
-    <t>10.0.2.120 - 10.0.2.199</t>
-  </si>
-  <si>
     <t>10.0.2.91</t>
   </si>
   <si>
@@ -193,13 +180,31 @@
   </si>
   <si>
     <t>10.0.2.183</t>
+  </si>
+  <si>
+    <t>Hole-RPSV PiHole (DNS Srv)</t>
+  </si>
+  <si>
+    <t>10.0.2.21 - 10.0.2.90</t>
+  </si>
+  <si>
+    <t>10.0.2.120 - 10.0.2.240</t>
+  </si>
+  <si>
+    <t>10.0.2.241 - 10.0.2.254</t>
+  </si>
+  <si>
+    <t># Hosts in RNG</t>
+  </si>
+  <si>
+    <t>&lt;- Total IPs in Range</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,6 +246,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -474,17 +488,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="double">
         <color auto="1"/>
@@ -550,11 +553,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="mediumDashed">
+        <color auto="1"/>
+      </right>
+      <top style="mediumDashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="mediumDashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -564,16 +582,15 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -596,12 +613,14 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -951,242 +970,272 @@
     <col min="3" max="3" width="24.5703125" customWidth="1"/>
     <col min="4" max="4" width="24.7109375" customWidth="1"/>
     <col min="5" max="5" width="23.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
     <col min="8" max="8" width="26.42578125" customWidth="1"/>
     <col min="9" max="9" width="60.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="G2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="42" t="s">
+      <c r="I2" s="40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="39" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="36" t="s">
+    <row r="4" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4">
+        <v>18</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="23">
         <v>1</v>
       </c>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="H3" s="40" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="41" t="s">
+      <c r="E5" s="24">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>69</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="21" t="s">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="26">
+        <v>1</v>
+      </c>
+      <c r="E6" s="27">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>8</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="29">
+        <v>1</v>
+      </c>
+      <c r="E7" s="30">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>19</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I7" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="29">
+        <v>2</v>
+      </c>
+      <c r="E8" s="30">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>120</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="32">
+        <v>0</v>
+      </c>
+      <c r="E9" s="33">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>13</v>
+      </c>
+      <c r="H9" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="24">
-        <v>1</v>
-      </c>
-      <c r="E5" s="25">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="27" t="s">
+    <row r="10" spans="2:9" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="27">
-        <v>1</v>
-      </c>
-      <c r="E6" s="28">
-        <v>0</v>
-      </c>
-      <c r="H6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="30">
-        <v>1</v>
-      </c>
-      <c r="E7" s="31">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="30" t="s">
+      <c r="C10" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="32">
+        <v>0</v>
+      </c>
+      <c r="E10" s="33">
+        <v>0</v>
+      </c>
+      <c r="G10" s="43">
+        <f>SUM(G3:G9)</f>
+        <v>248</v>
+      </c>
+      <c r="H10" s="42" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="32">
+        <v>0</v>
+      </c>
+      <c r="E11" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="30">
-        <v>2</v>
-      </c>
-      <c r="E8" s="31">
-        <v>1</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="32" t="s">
+      <c r="C12" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="32">
+        <v>0</v>
+      </c>
+      <c r="E12" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="32">
+        <v>0</v>
+      </c>
+      <c r="E13" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="32">
+        <v>0</v>
+      </c>
+      <c r="E14" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="33" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="33">
-        <v>0</v>
-      </c>
-      <c r="E9" s="34">
-        <v>0</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="33">
-        <v>0</v>
-      </c>
-      <c r="E10" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="33">
-        <v>0</v>
-      </c>
-      <c r="E11" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="33">
-        <v>0</v>
-      </c>
-      <c r="E12" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="33">
-        <v>0</v>
-      </c>
-      <c r="E13" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="33">
-        <v>0</v>
-      </c>
-      <c r="E14" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" s="33">
-        <v>0</v>
-      </c>
-      <c r="E15" s="34">
+      <c r="D15" s="32">
+        <v>0</v>
+      </c>
+      <c r="E15" s="33">
         <v>0</v>
       </c>
     </row>
@@ -1195,7 +1244,7 @@
         <v>8</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16" s="12">
         <v>0</v>
@@ -1206,10 +1255,10 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="D17" s="12">
         <v>0</v>
@@ -1220,10 +1269,10 @@
     </row>
     <row r="18" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="14" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" s="15">
         <v>1</v>

</xml_diff>

<commit_message>
Minor Style and Color Changes to TestLab IP Cfg
 Changes to be committed:
	modified:   TestLab IP Configuration.xlsx
    -Minor stylistic and color changes to the
	 tables in this file
</commit_message>
<xml_diff>
--- a/TestLab IP Configuration.xlsx
+++ b/TestLab IP Configuration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A5BDCE-BC53-4FFE-981D-6A319B84E0E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449354AC-D56B-4C63-95CA-38A5356095A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -256,7 +256,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -354,6 +354,16 @@
         </stop>
         <stop position="1">
           <color theme="8" tint="0.80001220740379042"/>
+        </stop>
+      </gradientFill>
+    </fill>
+    <fill>
+      <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
+        <stop position="0">
+          <color theme="4" tint="0.80001220740379042"/>
+        </stop>
+        <stop position="1">
+          <color theme="7"/>
         </stop>
       </gradientFill>
     </fill>
@@ -619,8 +629,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1161,11 +1171,11 @@
       <c r="E10" s="33">
         <v>0</v>
       </c>
-      <c r="G10" s="43">
+      <c r="G10" s="42">
         <f>SUM(G3:G9)</f>
         <v>248</v>
       </c>
-      <c r="H10" s="42" t="s">
+      <c r="H10" s="43" t="s">
         <v>54</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cleanup and Refinement of XLSX Style
</commit_message>
<xml_diff>
--- a/TestLab IP Configuration.xlsx
+++ b/TestLab IP Configuration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449354AC-D56B-4C63-95CA-38A5356095A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA245B63-B8C7-4B42-9638-6407CD1D0883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -194,10 +194,10 @@
     <t>10.0.2.241 - 10.0.2.254</t>
   </si>
   <si>
-    <t># Hosts in RNG</t>
-  </si>
-  <si>
     <t>&lt;- Total IPs in Range</t>
+  </si>
+  <si>
+    <t># of Hosts in IP Range</t>
   </si>
 </sst>
 </file>
@@ -980,7 +980,7 @@
     <col min="3" max="3" width="24.5703125" customWidth="1"/>
     <col min="4" max="4" width="24.7109375" customWidth="1"/>
     <col min="5" max="5" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" customWidth="1"/>
     <col min="8" max="8" width="26.42578125" customWidth="1"/>
     <col min="9" max="9" width="60.85546875" customWidth="1"/>
   </cols>
@@ -994,7 +994,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H2" s="40" t="s">
         <v>18</v>
@@ -1176,7 +1176,7 @@
         <v>248</v>
       </c>
       <c r="H10" s="43" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">

</xml_diff>